<commit_message>
added csv upload and appropriate error message on failure excel
</commit_message>
<xml_diff>
--- a/backend/shipping/data/success.xlsx
+++ b/backend/shipping/data/success.xlsx
@@ -23,13 +23,13 @@
     <t>Date</t>
   </si>
   <si>
-    <t>90001481754</t>
+    <t>90001483456</t>
   </si>
   <si>
-    <t>CR176752718888</t>
+    <t>CR176760825626</t>
   </si>
   <si>
-    <t>2026-01-04T14:09:05.659764834</t>
+    <t>2026-01-05T13:27:02.594868313</t>
   </si>
 </sst>
 </file>

</xml_diff>